<commit_message>
Finalize credential exclusions and verification notes
</commit_message>
<xml_diff>
--- a/reports/sales_en.xlsx
+++ b/reports/sales_en.xlsx
@@ -704,11 +704,11 @@
         <v>13</v>
       </c>
       <c r="B8" s="2">
-        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,A8)</f>
+        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A8,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>7</v>
       </c>
       <c r="C8" s="3">
-        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,A8)</f>
+        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A8,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>770.0</v>
       </c>
     </row>
@@ -717,11 +717,11 @@
         <v>15</v>
       </c>
       <c r="B9" s="2">
-        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,A9)</f>
+        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A9,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>9</v>
       </c>
       <c r="C9" s="3">
-        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,A9)</f>
+        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A9,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>675.0</v>
       </c>
     </row>
@@ -730,11 +730,11 @@
         <v>11</v>
       </c>
       <c r="B10" s="2">
-        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,A10)</f>
+        <f>SUMIFS('Sales'!D6:D11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A10,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>5</v>
       </c>
       <c r="C10" s="3">
-        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,A10)</f>
+        <f>SUMIFS('Sales'!F6:F11,'Sales'!C6:C11,"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(A10,"~","~~"),"*","~*"),"?","~?"))</f>
         <v>652.5</v>
       </c>
     </row>

</xml_diff>